<commit_message>
Add competitor intel, personalized draft emails, quick-log processor, as-built template
- Competitor Intel tab: 6 sourced metro Detroit incumbents with positioning
  and specific wedges against each; flags Wolverine Low Voltage as a
  possible subcontract channel (not just competition) and two unverified
  listings treated as unconfirmed.
- F.H. Paschen lead upgraded from paywalled-snippet evidence to primary-
  source confirmation (their own press release) with a named contact
  (Ken Swartz, VP) and real email -- first personalized Gmail draft created.
- New routine: quick-log processor (every 2h) turns a dictated "LOG:"
  email into a Pipeline update, so calls get logged without opening the
  spreadsheet.
- New AsBuilt_Documentation_Template.docx: TIA-606-structured job
  documentation to deliver with every completed job.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Metro_Detroit_Lead_Gen_System.xlsx
+++ b/Metro_Detroit_Lead_Gen_System.xlsx
@@ -13,6 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pipeline" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Call Rotation" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Events" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Competitor Intel" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4043,7 +4044,7 @@
         </is>
       </c>
       <c r="D35" s="27" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E35" s="28">
         <f>IFERROR(INDEX('Channel Performance'!$H$7:$H$16,MATCH(C35,'Channel Performance'!$A$7:$A$16,0)),1)</f>
@@ -4064,18 +4065,34 @@
       </c>
       <c r="I35" s="15" t="inlineStr">
         <is>
-          <t>Nearly tripling their Detroit office size right now — new/expanded space needs full cabling buildout, plus they're a construction firm that may sub out low-voltage on their own projects</t>
+          <t>Moved into new riverfront HQ (Talon Center) March 2, 2026, tripling Detroit office space — active buildout, plus actively hiring PM/Superintendent roles signaling growing project volume that may need low-voltage subs</t>
         </is>
       </c>
       <c r="J35" s="15" t="inlineStr">
         <is>
-          <t>Crain's Detroit Business, 2026: 'F.H. Paschen Contractors triples its Detroit office size' — Chicago-based infrastructure construction company, relocation fueled by business growth. crainsdetroit.com/real-estate/fh-paschen-contractors-triples-its-detroit-office-size — article itself is paywalled, confirm details before calling.</t>
-        </is>
-      </c>
-      <c r="K35" s="27" t="inlineStr"/>
-      <c r="L35" s="27" t="inlineStr"/>
-      <c r="M35" s="27" t="inlineStr"/>
-      <c r="N35" s="27" t="inlineStr"/>
+          <t>CONFIRMED via F.H. Paschen's own press release (primary source, not just news coverage): fhpaschen.com/f-h-paschen-triples-detroit-office-space-with-move-to-new-riverfront-headquarters — new address 100 River Place Drive, Suite 200 East, Detroit MI 48207; opened March 2, 2026; VP Ken Swartz leads the Detroit office; CEO quote confirms Detroit is a growth market; site also lists open PM/APM/Superintendent postings.</t>
+        </is>
+      </c>
+      <c r="K35" s="27" t="inlineStr">
+        <is>
+          <t>Ken Swartz (VP, Detroit office lead)</t>
+        </is>
+      </c>
+      <c r="L35" s="27" t="inlineStr">
+        <is>
+          <t>313-739-2123</t>
+        </is>
+      </c>
+      <c r="M35" s="27" t="inlineStr">
+        <is>
+          <t>kswartz@fhpaschen.com</t>
+        </is>
+      </c>
+      <c r="N35" s="27" t="inlineStr">
+        <is>
+          <t>fhpaschen.com</t>
+        </is>
+      </c>
       <c r="O35" s="29" t="inlineStr"/>
       <c r="P35" s="27" t="inlineStr">
         <is>
@@ -4084,13 +4101,13 @@
       </c>
       <c r="Q35" s="15" t="inlineStr">
         <is>
-          <t>Call: ask for facilities/office manager re: new space cabling; separately ask if they sub out low-voltage on their build projects</t>
+          <t>A draft email is waiting in your Gmail Drafts folder addressed to kswartz@fhpaschen.com — fill in [Your Name]/[Your Business Name]/[Your Phone] and review before sending. Update Status to Contacted once you actually send it.</t>
         </is>
       </c>
       <c r="R35" s="29" t="inlineStr"/>
       <c r="S35" s="15" t="inlineStr">
         <is>
-          <t>STRONG evidence — real, dated, specific physical-office-expansion signal, not a category guess. Read the full Crain's article yourself first (paywalled from here) to get the address/timeline before calling.</t>
+          <t>STRONGEST evidence in the pipeline — primary-source confirmation, named contact with real email, and a dual angle (their own office buildout + potential subcontract pipeline from their growth). Prioritize this one.</t>
         </is>
       </c>
     </row>
@@ -4135,13 +4152,21 @@
       </c>
       <c r="J36" s="24" t="inlineStr">
         <is>
-          <t>Crain's Detroit Business, 2026: 'Gardner White moving HQ from Warren to Bloomfield Hills in old Taubman building' — described as one of the more significant household-name relocations in metro Detroit recently. crainsdetroit.com/real-estate/commercial/cdb-gardner-white-moving-hq-20260625 — article paywalled, confirm timeline/scope before calling.</t>
+          <t>Crain's Detroit Business, 2026: 'Gardner White moving HQ from Warren to Bloomfield Hills in old Taubman building' — described as one of the more significant household-name relocations in metro Detroit recently. crainsdetroit.com/real-estate/commercial/cdb-gardner-white-moving-hq-20260625 — article paywalled, confirm timeline/scope before calling. Corporate/customer contact numbers confirmed via gardner-white.com but no named facilities/real estate contact found.</t>
         </is>
       </c>
       <c r="K36" s="25" t="inlineStr"/>
-      <c r="L36" s="20" t="inlineStr"/>
+      <c r="L36" s="20" t="inlineStr">
+        <is>
+          <t>586-774-8853 (corporate main line)</t>
+        </is>
+      </c>
       <c r="M36" s="25" t="inlineStr"/>
-      <c r="N36" s="20" t="inlineStr"/>
+      <c r="N36" s="20" t="inlineStr">
+        <is>
+          <t>gardner-white.com</t>
+        </is>
+      </c>
       <c r="O36" s="26" t="inlineStr"/>
       <c r="P36" s="20" t="inlineStr">
         <is>
@@ -4150,13 +4175,13 @@
       </c>
       <c r="Q36" s="12" t="inlineStr">
         <is>
-          <t>Read full article for move timeline, then call re: new HQ network/cabling buildout</t>
+          <t>Read full Crain's article for move timeline, then call corporate main line and ask specifically for facilities/real estate department re: new HQ buildout</t>
         </is>
       </c>
       <c r="R36" s="26" t="inlineStr"/>
       <c r="S36" s="12" t="inlineStr">
         <is>
-          <t>STRONG evidence — well-known local retailer (furniture), full HQ move = certain need for infrastructure work. Large enough that a GC/electrical contractor is likely already engaged — worth asking who that is too.</t>
+          <t>STRONG evidence — well-known local retailer (furniture), full HQ move = certain need for infrastructure work. Large enough that a GC/electrical contractor is likely already engaged — worth asking who that is too. No named contact yet, so this is a phone call, not an email draft.</t>
         </is>
       </c>
     </row>
@@ -11136,4 +11161,340 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Competitor Intel — Metro Detroit Cabling/Low-Voltage Incumbents</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="40" customHeight="1">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Real, sourced competitors in your 30-mile radius. Weekly refresh checks for hiring/news signals (a competitor hiring = busy = referral opportunity when they're overloaded; a competitor NOT hiring while you see market activity = they may be sitting on capacity, worth watching pricing).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>HQ / Coverage</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Size (sourced)</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Positioning (their own claim)</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>Their Strength</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>Your Wedge Against Them</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>Last Checked</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="70" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>T-Tech Solutions</t>
+        </is>
+      </c>
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>Troy, MI (HQ) + Rochester, Livonia, Utica, St. Clair Shores</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="inlineStr">
+        <is>
+          <t>16 employees, ~$6M revenue, founded 2008, 4.9★/55 reviews</t>
+        </is>
+      </c>
+      <c r="D6" s="12" t="inlineStr">
+        <is>
+          <t>Broad business/IT services provider — cabling is one of many offerings (also web dev, staffing, managed IT)</t>
+        </is>
+      </c>
+      <c r="E6" s="12" t="inlineStr">
+        <is>
+          <t>Multi-location scale, strong review volume, established since 2008, staffing arm gives them labor flexibility</t>
+        </is>
+      </c>
+      <c r="F6" s="12" t="inlineStr">
+        <is>
+          <t>They're a generalist IT shop, not a cabling specialist — you can out-focus them on cabling craft/documentation quality. Their breadth is also their dilution: small cabling jobs likely aren't their priority deal size.</t>
+        </is>
+      </c>
+      <c r="G6" s="12" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="H6" s="12" t="inlineStr">
+        <is>
+          <t>birdeye.com/t-tech-solutions, ttechsolutions.net, (248) 616-9600</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="70" customHeight="1">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>Wolverine Low Voltage</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="inlineStr">
+        <is>
+          <t>Ann Arbor, MI — services the full Lower Peninsula</t>
+        </is>
+      </c>
+      <c r="C7" s="15" t="inlineStr">
+        <is>
+          <t>Founded 2021 (young), team size not published</t>
+        </is>
+      </c>
+      <c r="D7" s="15" t="inlineStr">
+        <is>
+          <t>Full-stack: structured cabling, networking, cameras, access control, alarms</t>
+        </is>
+      </c>
+      <c r="E7" s="15" t="inlineStr">
+        <is>
+          <t>Broad service stack already matches your long-term vision; positive reviews on communication/project management</t>
+        </is>
+      </c>
+      <c r="F7" s="15" t="inlineStr">
+        <is>
+          <t>Young company (2021) — less entrenched than it looks. IMPORTANT: their own site says they 'partner with local businesses and individuals looking for work' — this may be a subcontract CHANNEL for you, not just a competitor. Worth a call to ask directly.</t>
+        </is>
+      </c>
+      <c r="G7" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="H7" s="15" t="inlineStr">
+        <is>
+          <t>wolverinelowvoltage.com/careers, wolverinelowvoltage.com/about-us</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="70" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>CTC Technologies</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>Ann Arbor, MI + Denver, CO</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="inlineStr">
+        <is>
+          <t>5★/10 reviews</t>
+        </is>
+      </c>
+      <c r="D8" s="12" t="inlineStr">
+        <is>
+          <t>Full IT solutions provider; structured cabling positioned as one solution among many, emphasizes fast response times</t>
+        </is>
+      </c>
+      <c r="E8" s="12" t="inlineStr">
+        <is>
+          <t>Explicitly competes on the same 'speed/responsiveness' wedge you were planning to use — they already claim 'industry-leading response times'</t>
+        </is>
+      </c>
+      <c r="F8" s="12" t="inlineStr">
+        <is>
+          <t>Their claim is marketing copy, not proof — a solo op who actually answers the phone and shows up same-day can out-execute a company-wide claim in practice. Don't concede the speed wedge just because they say it first; win it in practice.</t>
+        </is>
+      </c>
+      <c r="G8" s="12" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="H8" s="12" t="inlineStr">
+        <is>
+          <t>ctctechnologies.com/structured-cabling, birdeye.com/ctc-technologies-inc</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="70" customHeight="1">
+      <c r="A9" s="15" t="inlineStr">
+        <is>
+          <t>Detroit Field Techs</t>
+        </is>
+      </c>
+      <c r="B9" s="15" t="inlineStr">
+        <is>
+          <t>Detroit, MI — serves SE Michigan</t>
+        </is>
+      </c>
+      <c r="C9" s="15" t="inlineStr">
+        <is>
+          <t>Size unknown — no independent reviews found</t>
+        </is>
+      </c>
+      <c r="D9" s="15" t="inlineStr">
+        <is>
+          <t>Structured cabling, fiber, wireless, A/V — broad marketing site covering many Metro Detroit suburbs individually (SEO-style city pages)</t>
+        </is>
+      </c>
+      <c r="E9" s="15" t="inlineStr">
+        <is>
+          <t>Heavy local SEO footprint — likely ranks well for 'cabling contractor [suburb]' searches</t>
+        </is>
+      </c>
+      <c r="F9" s="15" t="inlineStr">
+        <is>
+          <t>No independent (non-self-published) reviews found — can't verify this is a distinct crew vs. a marketing/lead-gen site reselling to subs. Worth checking BBB/Google reviews directly before treating as a real competitor with a track record.</t>
+        </is>
+      </c>
+      <c r="G9" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="H9" s="15" t="inlineStr">
+        <is>
+          <t>detroitfieldtechs.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="70" customHeight="1">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>Metro Detroit Network Installers</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>Listed coverage: Rochester Hills/Oakland County</t>
+        </is>
+      </c>
+      <c r="C10" s="12" t="inlineStr">
+        <is>
+          <t>Unverified</t>
+        </is>
+      </c>
+      <c r="D10" s="12" t="inlineStr">
+        <is>
+          <t>Generic low-voltage/network installer marketing</t>
+        </is>
+      </c>
+      <c r="E10" s="12" t="inlineStr">
+        <is>
+          <t>Unknown — no independent verification found</t>
+        </is>
+      </c>
+      <c r="F10" s="12" t="inlineStr">
+        <is>
+          <t>Same caution as Detroit Field Techs — could not verify this is a distinct operating company vs. a directory/lead-gen listing. Don't assume it's a serious competitor without more digging.</t>
+        </is>
+      </c>
+      <c r="G10" s="12" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="H10" s="12" t="inlineStr">
+        <is>
+          <t>found via general web search, Aug 2026 — not independently verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="70" customHeight="1">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>US Cabling Pros</t>
+        </is>
+      </c>
+      <c r="B11" s="15" t="inlineStr">
+        <is>
+          <t>Listed coverage: Michigan, incl. Rochester Hills/Oakland County</t>
+        </is>
+      </c>
+      <c r="C11" s="15" t="inlineStr">
+        <is>
+          <t>Unverified</t>
+        </is>
+      </c>
+      <c r="D11" s="15" t="inlineStr">
+        <is>
+          <t>Generic low-voltage/network cabling marketing</t>
+        </is>
+      </c>
+      <c r="E11" s="15" t="inlineStr">
+        <is>
+          <t>Unknown — no independent verification found</t>
+        </is>
+      </c>
+      <c r="F11" s="15" t="inlineStr">
+        <is>
+          <t>Same caution as above — unverified. Treat as a placeholder until confirmed real with independent reviews or a physical presence.</t>
+        </is>
+      </c>
+      <c r="G11" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="H11" s="15" t="inlineStr">
+        <is>
+          <t>found via general web search, Aug 2026 — not independently verified</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>